<commit_message>
fixed code dublication from yolo_detector and table_manager
</commit_message>
<xml_diff>
--- a/data/outputs/table_status_report.xlsx
+++ b/data/outputs/table_status_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>00:00:15</t>
+          <t>00:00:01</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:00:01</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:00</t>
         </is>
       </c>
     </row>
@@ -507,7 +507,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -516,13 +516,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>00:00:08</t>
+          <t>00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -537,7 +537,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -546,20 +546,50 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:00:01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ready to order</t>
+          <t>need to clean</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>need to clean</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>00:00:00</t>
         </is>

</xml_diff>

<commit_message>
printing tables info in gui
</commit_message>
<xml_diff>
--- a/data/outputs/table_status_report.xlsx
+++ b/data/outputs/table_status_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,6 +445,261 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>00:00:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>00:00:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>00:00:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>00:00:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>00:00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ready to order</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>00:00:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ready to order</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>need to clean</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>00:00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>need to clean</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>00:00:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>eating</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>00:00:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>eating</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>00:00:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>need to clean</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>00:00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>need to clean</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>00:00:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>need to clean</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>00:00:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>need to clean</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>00:00:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>need to clean</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>00:00:11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added detect-set table mechanism still WIP
</commit_message>
<xml_diff>
--- a/data/outputs/table_status_report.xlsx
+++ b/data/outputs/table_status_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>00:00:10</t>
+          <t>00:00:03</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>00:00:10</t>
+          <t>00:00:03</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>00:00:08</t>
+          <t>00:00:00</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>00:00:10</t>
+          <t>00:00:02</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>00:00:04</t>
+          <t>00:00:02</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ready to order</t>
+          <t>available</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -546,157 +546,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>00:00:07</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ready to order</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
           <t>00:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>need to clean</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>00:00:01</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>need to clean</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>00:00:11</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>eating</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>00:00:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>eating</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>00:00:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>need to clean</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>00:00:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>need to clean</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>00:00:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>need to clean</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>00:00:11</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>need to clean</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>00:00:11</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>need to clean</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>00:00:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed set tables option
</commit_message>
<xml_diff>
--- a/data/outputs/table_status_report.xlsx
+++ b/data/outputs/table_status_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,22 +447,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>available</t>
+          <t>ready to order</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>00:00:03</t>
+          <t>00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -471,13 +471,13 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>00:00:03</t>
+          <t>00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -486,13 +486,13 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:00:10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -501,13 +501,13 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:12</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -516,13 +516,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -537,7 +537,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -546,7 +546,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>00:00:00</t>
+          <t>00:00:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>13</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>00:00:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
improved drawing design of labels and detections
</commit_message>
<xml_diff>
--- a/data/outputs/table_status_report.xlsx
+++ b/data/outputs/table_status_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,6 +445,111 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>00:00:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>00:00:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>00:00:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>00:00:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ready to order</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>00:00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>00:00:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added perfomance reviw and model selector
</commit_message>
<xml_diff>
--- a/data/outputs/table_status_report.xlsx
+++ b/data/outputs/table_status_report.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,111 +445,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>00:00:16</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>00:00:15</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>00:00:14</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>00:00:16</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ready to order</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>00:00:01</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>00:00:15</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>